<commit_message>
MHD - 20000, --num-walks 50 --walk-length 15 --p 3 --q 1
</commit_message>
<xml_diff>
--- a/results/MHD/node2vec_embedding_size_results.xlsx
+++ b/results/MHD/node2vec_embedding_size_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8338342357004563</v>
+        <v>0.8498324579153106</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8322792427232028</v>
+        <v>0.8473706462778301</v>
       </c>
     </row>
     <row r="4">
@@ -461,15 +461,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>0.8322424858955635</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>20</v>
-      </c>
-      <c r="B5" t="n">
-        <v>0.8226780457909166</v>
+        <v>0.8431637515113868</v>
       </c>
     </row>
   </sheetData>

</xml_diff>